<commit_message>
Performans zarfi kutle guncellemesi: 4S 13Ah AUW 4,0 kg (kullanici beyani), 3S 3,5 kg (varsayim); model ve tum tablolar/PNG'ler yeniden uretildi
</commit_message>
<xml_diff>
--- a/results/ucus_analiz_20260915/TABLOLAR/NAVITAS_ucus_analizi_tablolar.xlsx
+++ b/results/ucus_analiz_20260915/TABLOLAR/NAVITAS_ucus_analizi_tablolar.xlsx
@@ -2137,22 +2137,22 @@
         <v>11.4203</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>10.9498</v>
+        <v>11.3559</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>39.4</v>
+        <v>40.9</v>
       </c>
       <c r="K2" s="9" t="n">
-        <v>2.5916</v>
+        <v>2.7389</v>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 39 km/h)</t>
+          <t>✗ (asimptot 41 km/h)</t>
         </is>
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 39 km/h)</t>
+          <t>✗ (asimptot 41 km/h)</t>
         </is>
       </c>
       <c r="N2" s="9" t="n">
@@ -2214,22 +2214,22 @@
         <v>11.0141</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>10.6877</v>
+        <v>11.0797</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>38.5</v>
+        <v>39.9</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>2.6259</v>
+        <v>2.7737</v>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 38 km/h)</t>
+          <t>✗ (asimptot 40 km/h)</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 38 km/h)</t>
+          <t>✗ (asimptot 40 km/h)</t>
         </is>
       </c>
       <c r="N3" s="9" t="n">
@@ -2291,22 +2291,22 @@
         <v>8.630599999999999</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>9.044499999999999</v>
+        <v>9.3499</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>32.6</v>
+        <v>33.7</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>2.8594</v>
+        <v>3.0086</v>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 33 km/h)</t>
+          <t>✗ (asimptot 34 km/h)</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 33 km/h)</t>
+          <t>✗ (asimptot 34 km/h)</t>
         </is>
       </c>
       <c r="N4" s="9" t="n">
@@ -2370,20 +2370,20 @@
         <v>5.6619</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>61.9</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>5.5606</v>
-      </c>
-      <c r="L5" s="9" t="n">
-        <v>6.3366</v>
+        <v>6.4208</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>4.278</v>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 62 km/h)</t>
+          <t>✗ (asimptot 71 km/h)</t>
         </is>
       </c>
       <c r="N5" s="9" t="n">
@@ -2396,7 +2396,7 @@
         <v>41.1415</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="R5" s="11" t="n">
         <v>685.691</v>
@@ -2445,20 +2445,20 @@
         <v>5.6619</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>61.9</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>5.5606</v>
-      </c>
-      <c r="L6" s="9" t="n">
-        <v>6.3366</v>
+        <v>6.4208</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>4.278</v>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 62 km/h)</t>
+          <t>✗ (asimptot 71 km/h)</t>
         </is>
       </c>
       <c r="N6" s="9" t="n">
@@ -2471,7 +2471,7 @@
         <v>41.7176</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="R6" s="9" t="n">
         <v>695.2936999999999</v>
@@ -2520,20 +2520,20 @@
         <v>5.6619</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>61.9</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>5.5606</v>
-      </c>
-      <c r="L7" s="9" t="n">
-        <v>6.3366</v>
+        <v>6.4208</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>4.278</v>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 62 km/h)</t>
+          <t>✗ (asimptot 71 km/h)</t>
         </is>
       </c>
       <c r="N7" s="9" t="n">
@@ -2546,7 +2546,7 @@
         <v>45.5845</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>17.1873</v>
+        <v>19.8461</v>
       </c>
       <c r="R7" s="9" t="n">
         <v>759.7423</v>
@@ -2594,21 +2594,21 @@
       <c r="H8" s="9" t="n">
         <v>9.8066</v>
       </c>
-      <c r="I8" s="9" t="n">
-        <v>21.7372</v>
+      <c r="I8" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>78.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>4.0603</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <v>2.244</v>
+        <v>4.6884</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>2.0475</v>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 78 km/h)</t>
+          <t>✗ (asimptot 90 km/h)</t>
         </is>
       </c>
       <c r="N8" s="9" t="n">
@@ -2620,8 +2620,8 @@
       <c r="P8" s="11" t="n">
         <v>57.592</v>
       </c>
-      <c r="Q8" s="9" t="n">
-        <v>21.7372</v>
+      <c r="Q8" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="R8" s="9" t="n">
         <v>959.8668</v>
@@ -2669,21 +2669,21 @@
       <c r="H9" s="9" t="n">
         <v>9.8066</v>
       </c>
-      <c r="I9" s="9" t="n">
-        <v>21.7372</v>
+      <c r="I9" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>78.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>4.0603</v>
-      </c>
-      <c r="L9" s="11" t="n">
-        <v>2.244</v>
+        <v>4.6884</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>2.0475</v>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 78 km/h)</t>
+          <t>✗ (asimptot 90 km/h)</t>
         </is>
       </c>
       <c r="N9" s="9" t="n">
@@ -2695,8 +2695,8 @@
       <c r="P9" s="9" t="n">
         <v>58.4599</v>
       </c>
-      <c r="Q9" s="9" t="n">
-        <v>21.7372</v>
+      <c r="Q9" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="R9" s="9" t="n">
         <v>974.3313000000001</v>
@@ -2744,21 +2744,21 @@
       <c r="H10" s="9" t="n">
         <v>9.8066</v>
       </c>
-      <c r="I10" s="9" t="n">
-        <v>21.7372</v>
+      <c r="I10" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>78.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>4.0603</v>
-      </c>
-      <c r="L10" s="11" t="n">
-        <v>2.244</v>
+        <v>4.6884</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>2.0475</v>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 78 km/h)</t>
+          <t>✗ (asimptot 90 km/h)</t>
         </is>
       </c>
       <c r="N10" s="9" t="n">
@@ -2770,8 +2770,8 @@
       <c r="P10" s="9" t="n">
         <v>64.3719</v>
       </c>
-      <c r="Q10" s="9" t="n">
-        <v>21.7372</v>
+      <c r="Q10" s="10" t="n">
+        <v>25.1</v>
       </c>
       <c r="R10" s="9" t="n">
         <v>1072.8655</v>
@@ -2820,21 +2820,19 @@
         <v>15.6939</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>26.8095</v>
+        <v>30.9569</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>96.5</v>
+        <v>111.4</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>3.1292</v>
+        <v>3.6133</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>1.2431</v>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 97 km/h)</t>
-        </is>
+        <v>1.1872</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>2.8764</v>
       </c>
       <c r="N11" s="9" t="n">
         <v>126.3866</v>
@@ -2846,7 +2844,7 @@
         <v>96.16719999999999</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>26.8095</v>
+        <v>30.9569</v>
       </c>
       <c r="R11" s="9" t="n">
         <v>1602.7872</v>
@@ -2895,21 +2893,19 @@
         <v>15.6939</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>26.8095</v>
+        <v>30.9569</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>96.5</v>
+        <v>111.4</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>3.1292</v>
+        <v>3.6133</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>1.2431</v>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 97 km/h)</t>
-        </is>
+        <v>1.1872</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>2.8764</v>
       </c>
       <c r="N12" s="9" t="n">
         <v>123.9684</v>
@@ -2921,7 +2917,7 @@
         <v>97.9319</v>
       </c>
       <c r="Q12" s="9" t="n">
-        <v>26.8095</v>
+        <v>30.9569</v>
       </c>
       <c r="R12" s="9" t="n">
         <v>1632.1978</v>
@@ -2970,21 +2966,19 @@
         <v>15.6357</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>26.7597</v>
+        <v>30.8994</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>96.3</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>3.135</v>
+        <v>111.2</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>3.62</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>1.2487</v>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 96 km/h)</t>
-        </is>
+        <v>1.1922</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>2.8988</v>
       </c>
       <c r="N13" s="9" t="n">
         <v>109.7767</v>
@@ -3047,19 +3041,19 @@
         <v>19.3917</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>29.4642</v>
+        <v>34.0223</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>106.1</v>
+        <v>122.5</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>2.7832</v>
+        <v>3.2138</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.9741</v>
+        <v>0.9402</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>2.6777</v>
+        <v>2.0108</v>
       </c>
       <c r="N14" s="9" t="n">
         <v>126.3866</v>
@@ -3122,19 +3116,19 @@
         <v>19.0207</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>29.1809</v>
+        <v>33.6952</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>105.1</v>
-      </c>
-      <c r="K15" s="9" t="n">
-        <v>2.8103</v>
-      </c>
-      <c r="L15" s="11" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="M15" s="11" t="n">
-        <v>2.841</v>
+        <v>121.3</v>
+      </c>
+      <c r="K15" s="11" t="n">
+        <v>3.245</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>0.9605</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>2.0733</v>
       </c>
       <c r="N15" s="9" t="n">
         <v>123.9684</v>
@@ -3197,21 +3191,19 @@
         <v>16.8432</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>27.4599</v>
+        <v>31.7079</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>98.90000000000001</v>
+        <v>114.1</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>2.9864</v>
+        <v>3.4484</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>1.1479</v>
-      </c>
-      <c r="M16" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 99 km/h)</t>
-        </is>
+        <v>1.0996</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>2.5575</v>
       </c>
       <c r="N16" s="9" t="n">
         <v>109.7767</v>
@@ -3276,19 +3268,19 @@
         <v>21.2269</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>30.3794</v>
+        <v>35.0791</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>109.4</v>
+        <v>126.3</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>2.6216</v>
+        <v>3.0272</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.8822</v>
+        <v>0.8538</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>2.2233</v>
+        <v>1.7788</v>
       </c>
       <c r="N17" s="9" t="n">
         <v>126.3866</v>
@@ -3353,19 +3345,19 @@
         <v>20.8208</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>30.0874</v>
+        <v>34.7419</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>108.3</v>
-      </c>
-      <c r="K18" s="11" t="n">
-        <v>2.647</v>
+        <v>125.1</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>3.0565</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.9018</v>
+        <v>0.8721</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>2.3273</v>
+        <v>1.8311</v>
       </c>
       <c r="N18" s="9" t="n">
         <v>123.9684</v>
@@ -3430,19 +3422,19 @@
         <v>18.4372</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>28.3129</v>
+        <v>32.6929</v>
       </c>
       <c r="J19" s="10" t="n">
-        <v>101.9</v>
+        <v>117.7</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>2.8129</v>
+        <v>3.2481</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>1.0375</v>
+        <v>0.9973</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>3.5721</v>
+        <v>2.2252</v>
       </c>
       <c r="N19" s="9" t="n">
         <v>109.7767</v>
@@ -3508,7 +3500,7 @@
     <col width="14.6" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="24.05" customWidth="1" min="13" max="13"/>
     <col width="11.45" customWidth="1" min="14" max="14"/>
     <col width="19.85" customWidth="1" min="15" max="15"/>
     <col width="12.5" customWidth="1" min="16" max="16"/>
@@ -3654,22 +3646,22 @@
         <v>7.22</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>6.1407</v>
+        <v>6.3023</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>22.1</v>
+        <v>22.7</v>
       </c>
       <c r="K2" s="9" t="n">
-        <v>2.3923</v>
+        <v>2.4927</v>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 22 km/h)</t>
+          <t>✗ (asimptot 23 km/h)</t>
         </is>
       </c>
       <c r="M2" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 22 km/h)</t>
+          <t>✗ (asimptot 23 km/h)</t>
         </is>
       </c>
       <c r="N2" s="9" t="n">
@@ -3731,22 +3723,22 @@
         <v>6.8986</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>5.9371</v>
+        <v>6.0901</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>21.4</v>
+        <v>21.9</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>2.4239</v>
+        <v>2.5237</v>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 21 km/h)</t>
+          <t>✗ (asimptot 22 km/h)</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 21 km/h)</t>
+          <t>✗ (asimptot 22 km/h)</t>
         </is>
       </c>
       <c r="N3" s="9" t="n">
@@ -3808,13 +3800,13 @@
         <v>4.6001</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>4.3494</v>
-      </c>
-      <c r="J4" s="10" t="n">
-        <v>15.7</v>
+        <v>4.4404</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>16</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>2.6942</v>
+        <v>2.7852</v>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
@@ -3887,22 +3879,20 @@
         <v>5.6619</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>56.5</v>
+        <v>66.8</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>5.0761</v>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 56 km/h)</t>
-        </is>
+        <v>6.0061</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>4.7892</v>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 56 km/h)</t>
+          <t>✗ (asimptot 67 km/h)</t>
         </is>
       </c>
       <c r="N5" s="9" t="n">
@@ -3915,7 +3905,7 @@
         <v>34.9197</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="R5" s="9" t="n">
         <v>581.9954</v>
@@ -3964,22 +3954,20 @@
         <v>5.6619</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>56.5</v>
+        <v>66.8</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>5.0761</v>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 56 km/h)</t>
-        </is>
+        <v>6.0061</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>4.7892</v>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 56 km/h)</t>
+          <t>✗ (asimptot 67 km/h)</t>
         </is>
       </c>
       <c r="N6" s="9" t="n">
@@ -3992,7 +3980,7 @@
         <v>35.4589</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="R6" s="9" t="n">
         <v>590.9819</v>
@@ -4041,22 +4029,20 @@
         <v>5.6619</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>56.5</v>
+        <v>66.8</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>5.0761</v>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 56 km/h)</t>
-        </is>
+        <v>6.0061</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>4.7892</v>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 56 km/h)</t>
+          <t>✗ (asimptot 67 km/h)</t>
         </is>
       </c>
       <c r="N7" s="9" t="n">
@@ -4069,7 +4055,7 @@
         <v>40.1012</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>15.6898</v>
+        <v>18.5644</v>
       </c>
       <c r="R7" s="9" t="n">
         <v>668.3537</v>
@@ -4118,20 +4104,20 @@
         <v>9.8066</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>71.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>3.7065</v>
+        <v>4.3856</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>2.4704</v>
+        <v>2.1234</v>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 71 km/h)</t>
+          <t>✗ (asimptot 85 km/h)</t>
         </is>
       </c>
       <c r="N8" s="9" t="n">
@@ -4144,7 +4130,7 @@
         <v>50.0807</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="R8" s="9" t="n">
         <v>834.6789</v>
@@ -4193,20 +4179,20 @@
         <v>9.8066</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>71.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>3.7065</v>
+        <v>4.3856</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>2.4704</v>
+        <v>2.1234</v>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 71 km/h)</t>
+          <t>✗ (asimptot 85 km/h)</t>
         </is>
       </c>
       <c r="N9" s="9" t="n">
@@ -4219,7 +4205,7 @@
         <v>50.969</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="R9" s="9" t="n">
         <v>849.4835</v>
@@ -4268,20 +4254,20 @@
         <v>9.8066</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>71.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>3.7065</v>
+        <v>4.3856</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>2.4704</v>
+        <v>2.1234</v>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 71 km/h)</t>
+          <t>✗ (asimptot 85 km/h)</t>
         </is>
       </c>
       <c r="N10" s="9" t="n">
@@ -4294,7 +4280,7 @@
         <v>58.9879</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>19.8433</v>
+        <v>23.4789</v>
       </c>
       <c r="R10" s="11" t="n">
         <v>983.131</v>
@@ -4343,20 +4329,20 @@
         <v>14.4395</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>23.4751</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>84.5</v>
-      </c>
-      <c r="K11" s="11" t="n">
-        <v>2.978</v>
+        <v>27.7761</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>3.5237</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>1.4423</v>
+        <v>1.3335</v>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 85 km/h)</t>
+          <t>✗ (asimptot 100 km/h)</t>
         </is>
       </c>
       <c r="N11" s="9" t="n">
@@ -4420,20 +4406,20 @@
         <v>14.1668</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>23.2525</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>83.7</v>
+        <v>27.5127</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>99</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>3.0066</v>
+        <v>3.5574</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>1.4788</v>
+        <v>1.3638</v>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 84 km/h)</t>
+          <t>✗ (asimptot 99 km/h)</t>
         </is>
       </c>
       <c r="N12" s="9" t="n">
@@ -4496,21 +4482,21 @@
       <c r="H13" s="9" t="n">
         <v>12.2176</v>
       </c>
-      <c r="I13" s="9" t="n">
-        <v>21.5937</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>77.7</v>
+      <c r="I13" s="12" t="n">
+        <v>25.55</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>92</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>3.2375</v>
+        <v>3.8307</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>1.8113</v>
+        <v>1.6297</v>
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 78 km/h)</t>
+          <t>✗ (asimptot 92 km/h)</t>
         </is>
       </c>
       <c r="N13" s="9" t="n">
@@ -4574,21 +4560,19 @@
         <v>15.5547</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>24.0894</v>
+        <v>28.5029</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>86.7</v>
+        <v>102.6</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>2.8369</v>
+        <v>3.3566</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>1.3188</v>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 87 km/h)</t>
-        </is>
+        <v>1.2271</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>3.9871</v>
       </c>
       <c r="N14" s="9" t="n">
         <v>75.4706</v>
@@ -4651,21 +4635,19 @@
         <v>15.261</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>23.8609</v>
+        <v>28.2326</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>85.90000000000001</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>2.864</v>
+        <v>101.6</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>3.3888</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>1.3514</v>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 86 km/h)</t>
-        </is>
+        <v>1.2546</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>4.4524</v>
       </c>
       <c r="N15" s="9" t="n">
         <v>74.0458</v>
@@ -4728,20 +4710,20 @@
         <v>13.1612</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>22.1587</v>
+        <v>26.2185</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="K16" s="11" t="n">
-        <v>3.084</v>
+        <v>94.40000000000001</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>3.6491</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>1.6464</v>
+        <v>1.4959</v>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 80 km/h)</t>
+          <t>✗ (asimptot 94 km/h)</t>
         </is>
       </c>
       <c r="N16" s="9" t="n">
@@ -4807,21 +4789,19 @@
         <v>17.0267</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>24.8377</v>
+        <v>29.3883</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>89.40000000000001</v>
+        <v>105.8</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>2.6721</v>
+        <v>3.1617</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>1.1854</v>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 89 km/h)</t>
-        </is>
+        <v>1.1103</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>3.0804</v>
       </c>
       <c r="N17" s="9" t="n">
         <v>75.4706</v>
@@ -4886,21 +4866,19 @@
         <v>16.7052</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>24.6021</v>
+        <v>29.1096</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>88.59999999999999</v>
-      </c>
-      <c r="K18" s="9" t="n">
-        <v>2.6977</v>
+        <v>104.8</v>
+      </c>
+      <c r="K18" s="11" t="n">
+        <v>3.192</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>1.2141</v>
-      </c>
-      <c r="M18" s="6" t="inlineStr">
-        <is>
-          <t>✗ (asimptot 89 km/h)</t>
-        </is>
+        <v>1.1349</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>3.2712</v>
       </c>
       <c r="N18" s="9" t="n">
         <v>74.0458</v>
@@ -4964,21 +4942,21 @@
       <c r="H19" s="9" t="n">
         <v>14.4068</v>
       </c>
-      <c r="I19" s="11" t="n">
-        <v>22.847</v>
+      <c r="I19" s="9" t="n">
+        <v>27.0329</v>
       </c>
       <c r="J19" s="10" t="n">
-        <v>82.2</v>
+        <v>97.3</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>2.9049</v>
+        <v>3.4372</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>1.4711</v>
+        <v>1.3499</v>
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>✗ (asimptot 82 km/h)</t>
+          <t>✗ (asimptot 97 km/h)</t>
         </is>
       </c>
       <c r="N19" s="9" t="n">
@@ -5130,10 +5108,10 @@
         <v>62.4843</v>
       </c>
       <c r="F2" s="9" t="n">
-        <v>29.1648</v>
+        <v>33.6766</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>104.9933</v>
+        <v>121.2358</v>
       </c>
       <c r="H2" s="9" t="n">
         <v>126.3866</v>
@@ -5174,10 +5152,10 @@
         <v>61.9005</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>28.8307</v>
+        <v>33.2908</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>103.7904</v>
+        <v>119.8469</v>
       </c>
       <c r="H3" s="9" t="n">
         <v>123.9684</v>
@@ -5217,11 +5195,11 @@
       <c r="E4" s="9" t="n">
         <v>57.8665</v>
       </c>
-      <c r="F4" s="11" t="n">
-        <v>26.746</v>
+      <c r="F4" s="9" t="n">
+        <v>30.8836</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>96.2855</v>
+        <v>111.1809</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>109.7767</v>
@@ -5262,10 +5240,10 @@
         <v>54.8333</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>23.1728</v>
+        <v>27.4185</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>83.4222</v>
+        <v>98.70650000000001</v>
       </c>
       <c r="H5" s="9" t="n">
         <v>75.4706</v>
@@ -5306,10 +5284,10 @@
         <v>54.0527</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>22.8737</v>
+        <v>27.0646</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>82.3455</v>
+        <v>97.4325</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>74.0458</v>
@@ -5350,10 +5328,10 @@
         <v>47.1019</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>20.4893</v>
+        <v>24.2433</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>73.7615</v>
+        <v>87.2758</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>63.8579</v>
@@ -5764,7 +5742,7 @@
         </is>
       </c>
       <c r="C19" s="13" t="n">
-        <v>2.47853e-05</v>
+        <v>1.84934e-05</v>
       </c>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
@@ -5783,10 +5761,10 @@
       </c>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
@@ -6300,11 +6278,11 @@
         </is>
       </c>
       <c r="C44" s="6" t="n"/>
-      <c r="D44" s="12" t="n">
-        <v>29.42</v>
+      <c r="D44" s="9" t="n">
+        <v>39.2266</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>24.5166</v>
+        <v>34.3233</v>
       </c>
       <c r="F44" s="6" t="inlineStr"/>
     </row>
@@ -6419,10 +6397,10 @@
       </c>
       <c r="C50" s="6" t="n"/>
       <c r="D50" s="13" t="n">
-        <v>4.84873e-07</v>
+        <v>6.46498e-07</v>
       </c>
       <c r="E50" s="13" t="n">
-        <v>6.01855e-07</v>
+        <v>8.42598e-07</v>
       </c>
       <c r="F50" s="6" t="inlineStr"/>
     </row>
@@ -6478,11 +6456,11 @@
         </is>
       </c>
       <c r="C53" s="6" t="n"/>
-      <c r="D53" s="11" t="n">
-        <v>7.355</v>
+      <c r="D53" s="9" t="n">
+        <v>9.8066</v>
       </c>
       <c r="E53" s="9" t="n">
-        <v>6.1292</v>
+        <v>8.5808</v>
       </c>
       <c r="F53" s="6" t="inlineStr"/>
     </row>
@@ -6744,8 +6722,8 @@
         </is>
       </c>
       <c r="C67" s="6" t="n"/>
-      <c r="D67" s="11" t="n">
-        <v>14.048</v>
+      <c r="D67" s="9" t="n">
+        <v>18.7307</v>
       </c>
       <c r="E67" s="6" t="n"/>
       <c r="F67" s="6" t="inlineStr"/>
@@ -6901,7 +6879,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>4S T/W = 1,91 hava direnci ihmal edilmiş ALT SINIRDIR (E_1240_ivme/ozet.json: ivme tepesi t0+0,5 s'de hız ≈ 2,2 m/s → sürükleme ½ρ·CdA(0)·v² = 0,22 N = W'nin %0,8'i; tepe hız 5,20 m/s'de 1,24 N = %4,2). Tablolar bu alt sınıra kalibre olduğundan itki türevli sayılar (T_max/W, θ_max, a0) da alt sınırdır.</t>
+          <t>4S T/W = 1,91 hava direnci ihmal edilmiş ALT SINIRDIR (E_1240_ivme/ozet.json: ivme tepesi t0+0,5 s'de hız ≈ 2,2 m/s → sürükleme ½ρ·CdA(0)·v² = 0,22 N = W'nin %0,6'i; tepe hız 5,20 m/s'de 1,24 N = %3,2). Tablolar bu alt sınıra kalibre olduğundan itki türevli sayılar (T_max/W, θ_max, a0) da alt sınırdır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yuk-aski gazi tablosu (4S 13Ah, AUW 4,0 kg): xlsx sayfasi Y_Yuk_Aski_Gazi + png 46 + uretici betik
</commit_message>
<xml_diff>
--- a/results/ucus_analiz_20260915/TABLOLAR/NAVITAS_ucus_analizi_tablolar.xlsx
+++ b/results/ucus_analiz_20260915/TABLOLAR/NAVITAS_ucus_analizi_tablolar.xlsx
@@ -53,6 +53,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_B_3S_Komsu_Kiyas" sheetId="44" state="visible" r:id="rId44"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_C_Ucus_Bazinda" sheetId="45" state="visible" r:id="rId45"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K_D_Pencereleri" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Y_Yuk_Aski_Gazi" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +68,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00000E+00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +88,12 @@
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +103,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDE4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,9 +140,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -147,6 +155,10 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1911,10 +1923,39 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Kaynak: results/ucus_analiz_20260915/ (RAPOR.md, performans_zarfi/tablolar.json, E_1240_ivme/ozet.json, F_1311_aski_4S_13Ah/ozet.json, parametre_zaman_cizgisi.md/.json, tum_loglar.json, A/B/C/D/E ozet.json) · üretim: TABLOLAR/tablolar_uret.py · sayılar kopyalandı, yeniden hesaplanmadı (tek istisna: km/h = m/s × 3,6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Y_Yuk_Aski_Gazi</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Eklenen yük → askı gazı/akım/uçuş süresi (4S 13 Ah + 9x5x3, AUW 4,0 kg)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>performans_zarfi/tablolar.json kalibrasyonu + yuk_aski_tablosu.py</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>18</v>
+      </c>
+      <c r="E49" t="n">
+        <v>9</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>46_Y_Yuk_Aski_Gazi.png</t>
         </is>
       </c>
     </row>
@@ -1965,6 +2006,7 @@
     <hyperlink ref="A44" location="'K_B_3S_Komsu_Kiyas'!A1" display="K_B_3S_Komsu_Kiyas"/>
     <hyperlink ref="A45" location="'K_C_Ucus_Bazinda'!A1" display="K_C_Ucus_Bazinda"/>
     <hyperlink ref="A46" location="'K_D_Pencereleri'!A1" display="K_D_Pencereleri"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -54355,6 +54397,690 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Y — 4S 13 Ah + 9x5x3: eklenen yük → askı gazı / akım / uçuş süresi (AUW 4,0 kg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Pil V_açık</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>AUW kg</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>eklenen yük kg</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>askı gazı ThO</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>askı akımı A</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>askı gücü W</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>V_yük V</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>%80 pil ile dk</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>hüküm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>522</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="H3" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F4" t="n">
+        <v>623</v>
+      </c>
+      <c r="G4" t="n">
+        <v>15.58</v>
+      </c>
+      <c r="H4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E5" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>730</v>
+      </c>
+      <c r="G5" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="H5" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E6" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>842</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E7" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="F7" t="n">
+        <v>959</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="H7" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E8" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1082</v>
+      </c>
+      <c r="G8" t="n">
+        <v>14.54</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E9" t="n">
+        <v>85</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1209</v>
+      </c>
+      <c r="G9" t="n">
+        <v>14.21</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>sınırda (0,55–0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E10" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1341</v>
+      </c>
+      <c r="G10" t="n">
+        <v>13.86</v>
+      </c>
+      <c r="H10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>sınırda (0,55–0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>16.8 (dolu 4,20 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="E11" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1477</v>
+      </c>
+      <c r="G11" t="n">
+        <v>13.47</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>tehlikeli (&gt;0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="E12" t="n">
+        <v>36</v>
+      </c>
+      <c r="F12" t="n">
+        <v>522</v>
+      </c>
+      <c r="G12" t="n">
+        <v>14.51</v>
+      </c>
+      <c r="H12" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E13" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="F13" t="n">
+        <v>623</v>
+      </c>
+      <c r="G13" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="H13" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E14" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>730</v>
+      </c>
+      <c r="G14" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="H14" t="n">
+        <v>12</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E15" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>842</v>
+      </c>
+      <c r="G15" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="H15" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>uygun</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E16" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="F16" t="n">
+        <v>959</v>
+      </c>
+      <c r="G16" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>sınırda (0,55–0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E17" t="n">
+        <v>82.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1082</v>
+      </c>
+      <c r="G17" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>sınırda (0,55–0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="E18" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1209</v>
+      </c>
+      <c r="G18" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="H18" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>tehlikeli (&gt;0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="E19" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1341</v>
+      </c>
+      <c r="G19" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>tehlikeli (&gt;0,70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>15.6 (F logu başı 3,90 V/hücre)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>125.3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1477</v>
+      </c>
+      <c r="G20" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>kalkamaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kaynak: performans_zarfi/tablolar.json kalibrasyonu (askı 0,36 @ 14,0 V / 37,3 A; tam gaz T/W 1,91 @ 12,36 V / 115 A); AUW 4,0 kg kullanıcı beyanı (15 Eyl); R_paket 30,4 mΩ; kapasite 13 Ah × %80. Ölçülen azami T/W 1,91 → azami AUW 7,6 kg (sarkmış pil), dolu pil modeli 8,5 kg. Hüküm eşikleri: ArduPilot askı gazı &gt;0,70 yetersiz pay.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>